<commit_message>
mirando comando de scrolleo
</commit_message>
<xml_diff>
--- a/cypress/fixtures/CaptAccionistas.xlsx
+++ b/cypress/fixtures/CaptAccionistas.xlsx
@@ -3615,8 +3615,8 @@
     </row>
     <row r="2">
       <c r="A2" s="7" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(""1_xriSLIwwVjPl8SPQz6HpPENpfWiztH_Avw6PdiYhY8"", ""'0 Cliente'!B2"")  &amp; ""001"""),"0101 1997 33037001")</f>
-        <v>0101 1997 33037001</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(""1_xriSLIwwVjPl8SPQz6HpPENpfWiztH_Avw6PdiYhY8"", ""'0 Cliente'!B2"")  &amp; ""001"""),"0101 1997 33074001")</f>
+        <v>0101 1997 33074001</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -3650,8 +3650,8 @@
       <c r="C3" s="10"/>
       <c r="D3" s="9"/>
       <c r="E3" s="11" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("SUBSTITUTE(IMPORTRANGE(""1_xriSLIwwVjPl8SPQz6HpPENpfWiztH_Avw6PdiYhY8"", ""'0 Cliente'!B2""), "" "", """") &amp; ""03"""),"010119973303703")</f>
-        <v>010119973303703</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("SUBSTITUTE(IMPORTRANGE(""1_xriSLIwwVjPl8SPQz6HpPENpfWiztH_Avw6PdiYhY8"", ""'0 Cliente'!B2""), "" "", """") &amp; ""03"""),"010119973307403")</f>
+        <v>010119973307403</v>
       </c>
       <c r="F3" s="9"/>
       <c r="G3" s="11"/>
@@ -36755,8 +36755,8 @@
       </c>
       <c r="N3" s="11" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("RIGHT(SUBSTITUTE(IMPORTRANGE(""1_xriSLIwwVjPl8SPQz6HpPENpfWiztH_Avw6PdiYhY8"", ""'0 Cliente'!B2""), "" "", """"), 9)
-"),"199733037")</f>
-        <v>199733037</v>
+"),"199733074")</f>
+        <v>199733074</v>
       </c>
       <c r="O3" s="11" t="s">
         <v>14</v>
@@ -53777,8 +53777,8 @@
       <c r="A2" s="8"/>
       <c r="B2" s="8" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("SUBSTITUTE(IMPORTRANGE(""1_xriSLIwwVjPl8SPQz6HpPENpfWiztH_Avw6PdiYhY8"", ""'0 Cliente'!B2""), "" "", """")
-&amp; ""02"""),"010119973303702")</f>
-        <v>010119973303702</v>
+&amp; ""02"""),"010119973307402")</f>
+        <v>010119973307402</v>
       </c>
       <c r="C2" s="8" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
metdo para descarga de imagenes
</commit_message>
<xml_diff>
--- a/cypress/fixtures/CaptAccionistas.xlsx
+++ b/cypress/fixtures/CaptAccionistas.xlsx
@@ -3562,6 +3562,7 @@
   <cols>
     <col customWidth="1" min="1" max="2" width="17.63"/>
     <col customWidth="1" min="5" max="5" width="15.75"/>
+    <col customWidth="1" min="7" max="7" width="16.75"/>
     <col customWidth="1" min="8" max="8" width="26.63"/>
   </cols>
   <sheetData>
@@ -3615,8 +3616,8 @@
     </row>
     <row r="2">
       <c r="A2" s="7" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(""1_xriSLIwwVjPl8SPQz6HpPENpfWiztH_Avw6PdiYhY8"", ""'0 Cliente'!B2"")  &amp; ""001"""),"0101 1997 33074001")</f>
-        <v>0101 1997 33074001</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(""1_xriSLIwwVjPl8SPQz6HpPENpfWiztH_Avw6PdiYhY8"", ""'0 Cliente'!B2"")  &amp; ""001"""),"0101 1997 33102001")</f>
+        <v>0101 1997 33102001</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -3645,16 +3646,16 @@
       <c r="Z2" s="6"/>
     </row>
     <row r="3">
-      <c r="A3" s="3"/>
+      <c r="A3" s="7" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("IMPORTRANGE(""1_xriSLIwwVjPl8SPQz6HpPENpfWiztH_Avw6PdiYhY8"", ""'0 Cliente'!B2"")  &amp; ""003"""),"0101 1997 33102003")</f>
+        <v>0101 1997 33102003</v>
+      </c>
       <c r="B3" s="10"/>
       <c r="C3" s="10"/>
       <c r="D3" s="9"/>
-      <c r="E3" s="11" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("SUBSTITUTE(IMPORTRANGE(""1_xriSLIwwVjPl8SPQz6HpPENpfWiztH_Avw6PdiYhY8"", ""'0 Cliente'!B2""), "" "", """") &amp; ""03"""),"010119973307403")</f>
-        <v>010119973307403</v>
-      </c>
+      <c r="E3" s="9"/>
       <c r="F3" s="9"/>
-      <c r="G3" s="11"/>
+      <c r="G3" s="9"/>
       <c r="H3" s="11" t="s">
         <v>13</v>
       </c>
@@ -36755,8 +36756,8 @@
       </c>
       <c r="N3" s="11" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("RIGHT(SUBSTITUTE(IMPORTRANGE(""1_xriSLIwwVjPl8SPQz6HpPENpfWiztH_Avw6PdiYhY8"", ""'0 Cliente'!B2""), "" "", """"), 9)
-"),"199733074")</f>
-        <v>199733074</v>
+"),"199733102")</f>
+        <v>199733102</v>
       </c>
       <c r="O3" s="11" t="s">
         <v>14</v>
@@ -53777,8 +53778,8 @@
       <c r="A2" s="8"/>
       <c r="B2" s="8" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("SUBSTITUTE(IMPORTRANGE(""1_xriSLIwwVjPl8SPQz6HpPENpfWiztH_Avw6PdiYhY8"", ""'0 Cliente'!B2""), "" "", """")
-&amp; ""02"""),"010119973307402")</f>
-        <v>010119973307402</v>
+&amp; ""02"""),"010119973310202")</f>
+        <v>010119973310202</v>
       </c>
       <c r="C2" s="8" t="s">
         <v>13</v>

</xml_diff>